<commit_message>
Add tagging to exercises
</commit_message>
<xml_diff>
--- a/data/full_exercise_sheet.xlsx
+++ b/data/full_exercise_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Documents\Work\Udamy\Build a Backend REST API with Python &amp; Django\backend-app-api\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2381CC11-761D-4B1D-A328-EB208714F279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97BBDDFB-91B5-4219-B940-5BBEEC8EABD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exercises" sheetId="1" r:id="rId1"/>

</xml_diff>